<commit_message>
Implemented Models, DTOs, Services, and API controllers to allow for CRUD opperations on other media types. (Albums, Books, Games, Songs)
</commit_message>
<xml_diff>
--- a/Project Backlog.xlsx
+++ b/Project Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aaron\Projects\Capstone\Task 3\d424-capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80306812-97D1-4707-B76F-EEC4CE16D2B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4C3AAA-C331-4F96-9A4D-139B71F74452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7770" yWindow="10690" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Features" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
   <si>
     <t>Feature Name</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>in progress</t>
   </si>
 </sst>
 </file>
@@ -603,6 +606,9 @@
       <c r="F8">
         <v>3</v>
       </c>
+      <c r="G8" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="9" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C9" t="s">

</xml_diff>

<commit_message>
set up the front end media creation forms
</commit_message>
<xml_diff>
--- a/Project Backlog.xlsx
+++ b/Project Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aaron\Projects\Capstone\Task 3\d424-capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4C3AAA-C331-4F96-9A4D-139B71F74452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63297C4-B7A6-4029-8DD9-3043A20D5067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="16920" windowHeight="9560" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Features" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="50">
   <si>
     <t>Feature Name</t>
   </si>
@@ -155,6 +155,27 @@
   </si>
   <si>
     <t>in progress</t>
+  </si>
+  <si>
+    <t>Change Media button to reflect media type</t>
+  </si>
+  <si>
+    <t>Clear form on submission</t>
+  </si>
+  <si>
+    <t>or redirect to home page or item view</t>
+  </si>
+  <si>
+    <t>Make Ratings out of 5</t>
+  </si>
+  <si>
+    <t>platforms are not working on page</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Add Labels to relevent details on the view page</t>
   </si>
 </sst>
 </file>
@@ -196,21 +217,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
@@ -246,8 +253,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}" name="Table2" displayName="Table2" ref="C4:F8" totalsRowShown="0">
-  <autoFilter ref="C4:F8" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}" name="Table2" displayName="Table2" ref="C4:F13" totalsRowShown="0">
+  <autoFilter ref="C4:F13" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{C957A081-536B-4105-ABF4-D9CEBC20B3B4}" name="BugName"/>
     <tableColumn id="2" xr3:uid="{4DDF700F-AFCE-42BB-832C-B66E767CBDB2}" name="Notes"/>
@@ -522,16 +529,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="C4:G15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="70.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" customWidth="1"/>
+    <col min="3" max="3" width="25.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="70.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>0</v>
       </c>
@@ -548,7 +555,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>7</v>
       </c>
@@ -565,7 +572,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>9</v>
       </c>
@@ -579,7 +586,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>8</v>
       </c>
@@ -593,7 +600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>16</v>
       </c>
@@ -610,7 +617,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
         <v>19</v>
       </c>
@@ -624,7 +631,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>21</v>
       </c>
@@ -638,7 +645,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>23</v>
       </c>
@@ -652,7 +659,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>25</v>
       </c>
@@ -666,7 +673,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>32</v>
       </c>
@@ -677,7 +684,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
         <v>33</v>
       </c>
@@ -688,7 +695,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
         <v>39</v>
       </c>
@@ -716,15 +723,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7915A79-E61D-465A-9A2D-C1F6C4290640}">
   <dimension ref="C4:F16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="81.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" customWidth="1"/>
+    <col min="4" max="4" width="81.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>3</v>
       </c>
@@ -738,7 +745,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>5</v>
       </c>
@@ -749,7 +756,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>28</v>
       </c>
@@ -760,7 +767,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>30</v>
       </c>
@@ -770,8 +777,11 @@
       <c r="E7">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>34</v>
       </c>
@@ -781,8 +791,39 @@
       <c r="E8">
         <v>5</v>
       </c>
-    </row>
-    <row r="16" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="3:6" x14ac:dyDescent="0.35">
       <c r="D16" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
Added approprate labels to the media view detials page
</commit_message>
<xml_diff>
--- a/Project Backlog.xlsx
+++ b/Project Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aaron\Projects\Capstone\Task 3\d424-capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63297C4-B7A6-4029-8DD9-3043A20D5067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D297FFB-AE9B-4F68-AFD6-9662C9928264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="760" yWindow="760" windowWidth="16920" windowHeight="9560" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="48">
   <si>
     <t>Feature Name</t>
   </si>
@@ -158,12 +158,6 @@
   </si>
   <si>
     <t>Change Media button to reflect media type</t>
-  </si>
-  <si>
-    <t>Clear form on submission</t>
-  </si>
-  <si>
-    <t>or redirect to home page or item view</t>
   </si>
   <si>
     <t>Make Ratings out of 5</t>
@@ -254,7 +248,14 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}" name="Table2" displayName="Table2" ref="C4:F13" totalsRowShown="0">
-  <autoFilter ref="C4:F13" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}"/>
+  <autoFilter ref="C4:F13" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}">
+    <filterColumn colId="3">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C5:F13">
+    <sortCondition ref="F4:F13"/>
+  </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{C957A081-536B-4105-ABF4-D9CEBC20B3B4}" name="BugName"/>
     <tableColumn id="2" xr3:uid="{4DDF700F-AFCE-42BB-832C-B66E767CBDB2}" name="Notes"/>
@@ -745,82 +746,83 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="3:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="E5">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="F5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="F6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E7">
         <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="3:6" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="3:6" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
-        <v>43</v>
+        <v>45</v>
+      </c>
+      <c r="F9" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>6</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C13" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="16" spans="3:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Adds an edit form, an analytics page, and a search page. Also includes a small amount of responsive design for mobile devices. All added features had back end services and controllers set up.
</commit_message>
<xml_diff>
--- a/Project Backlog.xlsx
+++ b/Project Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aaron\Projects\Capstone\Task 3\d424-capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D297FFB-AE9B-4F68-AFD6-9662C9928264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F50EBD-802B-4A30-A636-D38FD7D36002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="16920" windowHeight="9560" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-7770" yWindow="10690" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Features" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="47">
   <si>
     <t>Feature Name</t>
   </si>
@@ -136,9 +136,6 @@
     <t>The log in screen does not display an error when you sign in with incorrect credientilas</t>
   </si>
   <si>
-    <t>s</t>
-  </si>
-  <si>
     <t>The creation screen needs to be able to allow for image upload</t>
   </si>
   <si>
@@ -154,9 +151,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>in progress</t>
-  </si>
-  <si>
     <t>Change Media button to reflect media type</t>
   </si>
   <si>
@@ -170,6 +164,9 @@
   </si>
   <si>
     <t>Add Labels to relevent details on the view page</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -185,15 +182,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -201,17 +204,88 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -233,8 +307,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{431196B2-32B8-4CC6-9A72-2DC075CEE389}" name="Table1" displayName="Table1" ref="C4:G18" totalsRowShown="0">
-  <autoFilter ref="C4:G18" xr:uid="{431196B2-32B8-4CC6-9A72-2DC075CEE389}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{431196B2-32B8-4CC6-9A72-2DC075CEE389}" name="Table1" displayName="Table1" ref="C4:G15" totalsRowShown="0">
+  <autoFilter ref="C4:G15" xr:uid="{431196B2-32B8-4CC6-9A72-2DC075CEE389}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C5:G10">
+    <sortCondition ref="G4:G10"/>
+  </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{39000331-3D1D-473C-B7B6-078D66FD392A}" name="Feature Name"/>
     <tableColumn id="2" xr3:uid="{C8097EEA-8204-4B43-ABBE-6351FC44BE82}" name="Notes"/>
@@ -248,11 +325,7 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}" name="Table2" displayName="Table2" ref="C4:F13" totalsRowShown="0">
-  <autoFilter ref="C4:F13" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}">
-    <filterColumn colId="3">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="C4:F13" xr:uid="{1289C8C0-264A-4109-BD4A-4D61001AB2FE}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C5:F13">
     <sortCondition ref="F4:F13"/>
   </sortState>
@@ -529,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C4:G15"/>
+  <dimension ref="C4:R15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="25.54296875" bestFit="1" customWidth="1"/>
@@ -539,7 +612,7 @@
     <col min="7" max="7" width="12.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>0</v>
       </c>
@@ -556,7 +629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>7</v>
       </c>
@@ -570,74 +643,148 @@
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="3:7" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>2</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="P6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F6">
+      <c r="Q6" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="3:7" x14ac:dyDescent="0.35">
+      <c r="R6" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="3:7" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
+        <v>40</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2">
+        <v>5</v>
+      </c>
+      <c r="R7" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="3:7" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5">
+        <v>5</v>
+      </c>
+      <c r="R8" s="6"/>
+    </row>
+    <row r="9" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
         <v>12</v>
       </c>
       <c r="F9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="3:7" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+      <c r="G9" t="s">
+        <v>40</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2">
+        <v>5</v>
+      </c>
+      <c r="R9" s="3"/>
+    </row>
+    <row r="10" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E10" t="s">
         <v>12</v>
@@ -645,72 +792,91 @@
       <c r="F10">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="3:7" x14ac:dyDescent="0.35">
+      <c r="G10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="3:7" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+      <c r="G11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="E12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="3:7" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+      <c r="G12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F13">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="3:18" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
         <v>33</v>
       </c>
       <c r="D14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="3:18" x14ac:dyDescent="0.35">
+      <c r="C15" t="s">
         <v>38</v>
       </c>
-      <c r="F14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="3:7" x14ac:dyDescent="0.35">
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>39</v>
       </c>
-      <c r="D15" t="s">
-        <v>40</v>
-      </c>
       <c r="F15">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C4:G18">
-    <cfRule type="expression" dxfId="0" priority="1">
+  <conditionalFormatting sqref="C4:G15">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>$G4="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N6:R9">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>$G6="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N5:Q5">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>#REF!="Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -723,10 +889,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7915A79-E61D-465A-9A2D-C1F6C4290640}">
-  <dimension ref="C4:F16"/>
+  <dimension ref="C4:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="81.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.81640625" customWidth="1"/>
@@ -746,7 +912,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>28</v>
       </c>
@@ -757,10 +923,10 @@
         <v>5</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>30</v>
       </c>
@@ -771,10 +937,10 @@
         <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>34</v>
       </c>
@@ -785,23 +951,29 @@
         <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8">
+        <v>5</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C9" t="s">
         <v>43</v>
       </c>
-      <c r="F8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="3:6" hidden="1" x14ac:dyDescent="0.35">
-      <c r="C9" t="s">
-        <v>45</v>
+      <c r="E9">
+        <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="3:6" x14ac:dyDescent="0.35">
@@ -814,20 +986,30 @@
       <c r="E10">
         <v>5</v>
       </c>
+      <c r="F10" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
-        <v>44</v>
+        <v>42</v>
+      </c>
+      <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="D16" t="s">
-        <v>36</v>
+        <v>45</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>